<commit_message>
docs: perbarui mapping 1-to-1 pasti dari stockDetails ke Excel tanpa fallback chaining
</commit_message>
<xml_diff>
--- a/Dokumentasi_Spesifikasi_Mapping_Asset_Counting.xlsx
+++ b/Dokumentasi_Spesifikasi_Mapping_Asset_Counting.xlsx
@@ -13,15 +13,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="136">
-  <si>
-    <t>SPESIFIKASI MAPPING JSON KE EXCEL - FORM ASSET COUNTING</t>
-  </si>
-  <si>
-    <t>Dokumen acuan untuk System Analyst (SA) &amp; Backend Developer dalam integrasi data API Asset Counting.</t>
-  </si>
-  <si>
-    <t>A. METADATA HEADER (Bagian Atas Laporan)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="118">
+  <si>
+    <t>SPESIFIKASI MAPPING 1-TO-1 JSON KE EXCEL - FORM ASSET COUNTING</t>
+  </si>
+  <si>
+    <t>Dokumen acuan pasti 1-to-1 untuk System Analyst (SA) &amp; Backend Developer dari objek root dan array stockDetails.</t>
+  </si>
+  <si>
+    <t>A. METADATA HEADER (Root JSON Object)</t>
   </si>
   <si>
     <t>Posisi Sel Excel</t>
@@ -30,10 +30,7 @@
     <t>Teks di Excel</t>
   </si>
   <si>
-    <t>Field JSON Utama (BE)</t>
-  </si>
-  <si>
-    <t>Field JSON Alternatif</t>
+    <t>Field JSON Backend (Pasti)</t>
   </si>
   <si>
     <t>Tipe Data</t>
@@ -42,7 +39,7 @@
     <t>Contoh Nilai</t>
   </si>
   <si>
-    <t>Keterangan SA/BE</t>
+    <t>Keterangan</t>
   </si>
   <si>
     <t>Sel A1</t>
@@ -54,16 +51,13 @@
     <t>office_branch_name</t>
   </si>
   <si>
-    <t>office_name / branch_name / cabang</t>
-  </si>
-  <si>
     <t>String</t>
   </si>
   <si>
     <t>Biak</t>
   </si>
   <si>
-    <t>Nama cabang operasional. Huruf otomatis dikonversi ke UPPERCASE.</t>
+    <t>Nama cabang operasional (Otomatis UPPERCASE di Excel).</t>
   </si>
   <si>
     <t>Sel A2</t>
@@ -75,9 +69,6 @@
     <t>(Fixed Text)</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>Judul tetap laporan di baris 2.</t>
   </si>
   <si>
@@ -87,22 +78,19 @@
     <t>TAHUN BUKU [TAHUN]</t>
   </si>
   <si>
-    <t>fiscal_year</t>
-  </si>
-  <si>
-    <t>doc_date / periode_start / created_date</t>
-  </si>
-  <si>
-    <t>Integer / Date</t>
-  </si>
-  <si>
-    <t>2025</t>
-  </si>
-  <si>
-    <t>Tahun buku laporan. Jika tidak dikirim, diekstrak dari tahun doc_date atau tahun berjalan.</t>
-  </si>
-  <si>
-    <t>B. DETAIL 12 KOLOM TABEL ASET (Array: stockDetails / details)</t>
+    <t>doc_date</t>
+  </si>
+  <si>
+    <t>String (Date)</t>
+  </si>
+  <si>
+    <t>2025-11-18 09:03:54.000</t>
+  </si>
+  <si>
+    <t>Tahun buku diambil dari tahun doc_date (misal: 2025).</t>
+  </si>
+  <si>
+    <t>B. DETAIL 12 KOLOM TABEL ASET (Array: stockDetails)</t>
   </si>
   <si>
     <t>Kolom Excel</t>
@@ -111,31 +99,28 @@
     <t>Nama Kolom di Excel</t>
   </si>
   <si>
-    <t>Format / Transformasi di Excel</t>
-  </si>
-  <si>
     <t>Contoh Nilai JSON</t>
   </si>
   <si>
+    <t>Format &amp; Keterangan di Excel</t>
+  </si>
+  <si>
     <t>Kolom A</t>
   </si>
   <si>
     <t>NO</t>
   </si>
   <si>
-    <t>no</t>
-  </si>
-  <si>
-    <t>stockdetail_id / nomor urut</t>
+    <t>(Nomor Urut Iterasi)</t>
   </si>
   <si>
     <t>Integer</t>
   </si>
   <si>
-    <t>Nomor urut numerik (1, 2, 3, ...)</t>
-  </si>
-  <si>
-    <t>1</t>
+    <t>1, 2, 3, ...</t>
+  </si>
+  <si>
+    <t>Nomor urut baris di Excel (1, 2, 3, ...)</t>
   </si>
   <si>
     <t>Kolom B</t>
@@ -147,15 +132,12 @@
     <t>item_code</t>
   </si>
   <si>
-    <t>item_code_sap / serial / nomor_asset_modul</t>
-  </si>
-  <si>
-    <t>Teks kode aset dari sistem/SAP</t>
-  </si>
-  <si>
     <t>30200B9902001</t>
   </si>
   <si>
+    <t>Nomor / kode aset dari modul SAP</t>
+  </si>
+  <si>
     <t>Kolom C</t>
   </si>
   <si>
@@ -165,10 +147,7 @@
     <t>serial</t>
   </si>
   <si>
-    <t>nomor_asset_scan / item_code / barcode</t>
-  </si>
-  <si>
-    <t>Teks barcode scan (Cell Highlight Kuning #FFFF00)</t>
+    <t>Nomor barcode hasil scan fisik (Highlight Kuning #FFFF00)</t>
   </si>
   <si>
     <t>Kolom D</t>
@@ -180,15 +159,12 @@
     <t>item_name</t>
   </si>
   <si>
-    <t>nama_asset / asset_name / name</t>
-  </si>
-  <si>
-    <t>Deskripsi/nama aset fisik</t>
-  </si>
-  <si>
     <t>BANGUNAN</t>
   </si>
   <si>
+    <t>Nama / deskripsi barang aset</t>
+  </si>
+  <si>
     <t>Kolom E</t>
   </si>
   <si>
@@ -198,18 +174,12 @@
     <t>tanggal_perolehan</t>
   </si>
   <si>
-    <t>TanggalPerolehan / acquisition_date</t>
-  </si>
-  <si>
-    <t>Date / String</t>
-  </si>
-  <si>
-    <t>Format YYYY-MM-DD (timestamp jam dibuang)</t>
-  </si>
-  <si>
     <t>1993-10-21 00:00:00.000</t>
   </si>
   <si>
+    <t>Tanggal perolehan (Format YYYY-MM-DD, jam dibersihkan)</t>
+  </si>
+  <si>
     <t>Kolom F</t>
   </si>
   <si>
@@ -219,18 +189,15 @@
     <t>harga_perolehan</t>
   </si>
   <si>
-    <t>HargaPerolehan / acquisition_cost</t>
-  </si>
-  <si>
     <t>Number / String</t>
   </si>
   <si>
-    <t>Format Angka Mata Uang (#,##0)</t>
-  </si>
-  <si>
     <t>2696351206.000000</t>
   </si>
   <si>
+    <t>Harga beli perolehan (Format Angka #,##0)</t>
+  </si>
+  <si>
     <t>Kolom G</t>
   </si>
   <si>
@@ -240,15 +207,12 @@
     <t>akumulasi_penyusutan</t>
   </si>
   <si>
-    <t>AkumulasiPenyusutan / depreciation</t>
-  </si>
-  <si>
-    <t>Format Angka Mata Uang (#,##0). String ".000000" diubah ke 0</t>
-  </si>
-  <si>
     <t>.000000</t>
   </si>
   <si>
+    <t>Akumulasi depresiasi (Format Angka #,##0, .000000 -&gt; 0)</t>
+  </si>
+  <si>
     <t>Kolom H</t>
   </si>
   <si>
@@ -258,10 +222,7 @@
     <t>nbv</t>
   </si>
   <si>
-    <t>Nbv / (HargaPerolehan - AkumulasiPenyusutan)</t>
-  </si>
-  <si>
-    <t>Net Book Value / Nilai Buku (#,##0)</t>
+    <t>Net Book Value / Nilai Buku (Format Angka #,##0)</t>
   </si>
   <si>
     <t>Kolom I</t>
@@ -273,13 +234,10 @@
     <t>asset_pic</t>
   </si>
   <si>
-    <t>user_pengguna / pic / asset_location</t>
-  </si>
-  <si>
-    <t>Nama penanggung jawab atau lokasi fisik aset</t>
-  </si>
-  <si>
-    <t>Sunardi / (CAB. BIAK)</t>
+    <t>Sunardi</t>
+  </si>
+  <si>
+    <t>Nama PIC / pemegang aset (Jika null tampil -)</t>
   </si>
   <si>
     <t>Kolom J</t>
@@ -291,15 +249,12 @@
     <t>asset_condition</t>
   </si>
   <si>
-    <t>status_barang / is_checked</t>
-  </si>
-  <si>
-    <t>Kondisi barang (Cell Highlight Kuning #FFFF00, default: ADA)</t>
-  </si>
-  <si>
     <t>ADA</t>
   </si>
   <si>
+    <t>Status keberadaan barang (Highlight Kuning #FFFF00, default: ADA)</t>
+  </si>
+  <si>
     <t>Kolom K</t>
   </si>
   <si>
@@ -309,16 +264,13 @@
     <t>attachment</t>
   </si>
   <si>
-    <t>foto_unit / img_path / foto</t>
-  </si>
-  <si>
-    <t>Array / String</t>
-  </si>
-  <si>
-    <t>Foto di-embed otomatis (1-5 thumbnail rapi)</t>
-  </si>
-  <si>
-    <t>["https://hrms.hasjrat.co.id/horor/...jpg"]</t>
+    <t>Array [URL]</t>
+  </si>
+  <si>
+    <t>["https://.../foto1.jpg"]</t>
+  </si>
+  <si>
+    <t>Foto unit ter-embed rapi (1-5 foto per baris)</t>
   </si>
   <si>
     <t>Kolom L</t>
@@ -327,16 +279,13 @@
     <t>KETERANGAN</t>
   </si>
   <si>
-    <t>remarks</t>
-  </si>
-  <si>
-    <t>checked_remarks / asset_location / keterangan</t>
-  </si>
-  <si>
-    <t>Catatan tambahan / lokasi fisik</t>
+    <t>asset_location</t>
   </si>
   <si>
     <t>CAB. BIAK</t>
+  </si>
+  <si>
+    <t>Lokasi fisik / catatan aset di cabang</t>
   </si>
   <si>
     <t>PT HASJRAT ABADI CABANG BIAK</t>
@@ -356,7 +305,7 @@
     <t>1993-10-21</t>
   </si>
   <si>
-    <t>(CAB. BIAK)</t>
+    <t>-</t>
   </si>
   <si>
     <t>[Foto Unit Disematkan]</t>
@@ -375,9 +324,6 @@
   </si>
   <si>
     <t>2014-07-18</t>
-  </si>
-  <si>
-    <t>Sunardi</t>
   </si>
   <si>
     <t>30200K1502001</t>
@@ -436,15 +382,14 @@
       "serial": "30200B9902001",
       "asset_pic": "Sunardi",
       "asset_location": "CAB. BIAK",
-      "TanggalPerolehan": "1993-10-21 00:00:00.000",
-      "HargaPerolehan": "2696351206.000000",
-      "AkumulasiPenyusutan": ".000000",
-      "Nbv": "2696351206.000000",
+      "tanggal_perolehan": "1993-10-21 00:00:00.000",
+      "harga_perolehan": "2696351206.000000",
+      "akumulasi_penyusutan": ".000000",
+      "nbv": "2696351206.000000",
       "asset_condition": "ADA",
       "attachment": [
         "https://hrms.hasjrat.co.id/horor/hororupload/section/sample1.jpg"
-      ],
-      "remarks": "Kondisi fisik gedung baik"
+      ]
     }
   ]
 }</t>
@@ -1008,19 +953,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="24" customWidth="1"/>
-    <col min="4" max="4" width="34" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="38" customWidth="1"/>
-    <col min="7" max="7" width="28" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+    <col min="6" max="6" width="44" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1029,7 +973,6 @@
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1041,7 +984,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
@@ -1060,90 +1003,78 @@
       <c r="F5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="4" t="s">
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="C6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="6" t="s">
+    </row>
+    <row r="7" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="B7" s="8" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+      <c r="C7" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>19</v>
-      </c>
       <c r="D7" s="8" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F7" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="8" t="s">
+    </row>
+    <row r="8" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="8" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="E8" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="F8" s="6" t="s">
         <v>24</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>5</v>
@@ -1152,294 +1083,255 @@
         <v>6</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="F11" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="D12" s="10" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="12" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="9" t="s">
+      <c r="E12" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="F12" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="10" t="s">
+    </row>
+    <row r="13" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="B13" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="C13" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="D13" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="G12" s="10" t="s">
+      <c r="F13" s="12" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="13" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="11" t="s">
+    <row r="14" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B14" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C14" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D14" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="F14" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="E13" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="F13" s="12" t="s">
+    </row>
+    <row r="15" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="G13" s="12" t="s">
+      <c r="B15" s="12" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="14" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
+      <c r="C15" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="D15" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="F15" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="D14" s="10" t="s">
+    </row>
+    <row r="16" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="E14" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="F14" s="10" t="s">
+      <c r="B16" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="G14" s="10" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="15" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="11" t="s">
+      <c r="C16" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="D16" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="E16" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="F16" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="D15" s="12" t="s">
+    </row>
+    <row r="17" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="E15" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="F15" s="12" t="s">
+      <c r="B17" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="G15" s="12" t="s">
+      <c r="C17" s="12" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="16" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="9" t="s">
+      <c r="D17" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="E17" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="F17" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="D16" s="10" t="s">
+    </row>
+    <row r="18" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="B18" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="F16" s="10" t="s">
+      <c r="C18" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="G16" s="10" t="s">
+      <c r="D18" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="E18" s="10" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="17" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="11" t="s">
+      <c r="F18" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="B17" s="12" t="s">
+    </row>
+    <row r="19" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="B19" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="D17" s="12" t="s">
+      <c r="C19" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="E17" s="12" t="s">
+      <c r="D19" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="F19" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="F17" s="12" t="s">
+    </row>
+    <row r="20" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="G17" s="12" t="s">
+      <c r="B20" s="10" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="18" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="s">
+      <c r="C20" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="D20" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="F20" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="D18" s="10" t="s">
+    </row>
+    <row r="21" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="E18" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="F18" s="10" t="s">
+      <c r="B21" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="G18" s="10" t="s">
+      <c r="C21" s="12" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="19" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="11" t="s">
+      <c r="D21" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="B19" s="12" t="s">
+      <c r="F21" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="C19" s="12" t="s">
+    </row>
+    <row r="22" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="D19" s="12" t="s">
+      <c r="B22" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="E19" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="F19" s="12" t="s">
+      <c r="C22" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="G19" s="12" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="20" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="9" t="s">
+      <c r="D22" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="E22" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="F22" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="D20" s="10" t="s">
+    </row>
+    <row r="23" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="E20" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="F20" s="10" t="s">
+      <c r="B23" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="G20" s="10" t="s">
+      <c r="C23" s="12" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="21" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="11" t="s">
+      <c r="D23" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="F23" s="12" t="s">
         <v>90</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="D21" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="E21" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="F21" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="G21" s="12" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="22" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="B22" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="C22" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="D22" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="F22" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="G22" s="10" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="23" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="C23" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="D23" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="E23" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="F23" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="G23" s="12" t="s">
-        <v>107</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1465,56 +1357,56 @@
   <sheetData>
     <row r="1" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>108</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
-        <v>109</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" ht="28" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>111</v>
+        <v>94</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="I5" s="14" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="J5" s="14" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="K5" s="14" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="L5" s="14" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1522,16 +1414,16 @@
         <v>1</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>112</v>
+        <v>95</v>
       </c>
       <c r="F6" s="19">
         <v>2696351206</v>
@@ -1543,16 +1435,16 @@
         <v>2696351206</v>
       </c>
       <c r="I6" s="16" t="s">
-        <v>113</v>
+        <v>96</v>
       </c>
       <c r="J6" s="17" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="K6" s="16" t="s">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="L6" s="18" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1560,16 +1452,16 @@
         <v>2</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>20</v>
+        <v>96</v>
       </c>
       <c r="F7" s="19">
         <v>0</v>
@@ -1581,16 +1473,16 @@
         <v>0</v>
       </c>
       <c r="I7" s="16" t="s">
-        <v>113</v>
+        <v>96</v>
       </c>
       <c r="J7" s="17" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="K7" s="16" t="s">
-        <v>20</v>
+        <v>96</v>
       </c>
       <c r="L7" s="18" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1598,16 +1490,16 @@
         <v>3</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>118</v>
+        <v>101</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="F8" s="19">
         <v>10346600</v>
@@ -1619,16 +1511,16 @@
         <v>8406613</v>
       </c>
       <c r="I8" s="16" t="s">
-        <v>120</v>
+        <v>73</v>
       </c>
       <c r="J8" s="17" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="K8" s="16" t="s">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="L8" s="18" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1636,16 +1528,16 @@
         <v>4</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>121</v>
+        <v>103</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>121</v>
+        <v>103</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>20</v>
+        <v>96</v>
       </c>
       <c r="F9" s="19">
         <v>0</v>
@@ -1657,16 +1549,16 @@
         <v>0</v>
       </c>
       <c r="I9" s="16" t="s">
-        <v>113</v>
+        <v>96</v>
       </c>
       <c r="J9" s="17" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="K9" s="16" t="s">
-        <v>20</v>
+        <v>96</v>
       </c>
       <c r="L9" s="18" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1674,16 +1566,16 @@
         <v>5</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>20</v>
+        <v>96</v>
       </c>
       <c r="F10" s="19">
         <v>0</v>
@@ -1695,16 +1587,16 @@
         <v>0</v>
       </c>
       <c r="I10" s="16" t="s">
-        <v>113</v>
+        <v>96</v>
       </c>
       <c r="J10" s="17" t="s">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="K10" s="16" t="s">
-        <v>20</v>
+        <v>96</v>
       </c>
       <c r="L10" s="18" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -1725,7 +1617,7 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="20" t="s">
-        <v>125</v>
+        <v>107</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -1734,10 +1626,10 @@
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
-        <v>126</v>
+        <v>108</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>127</v>
+        <v>109</v>
       </c>
       <c r="C3" s="22"/>
       <c r="D3" s="22"/>
@@ -1745,10 +1637,10 @@
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="21" t="s">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="C4" s="22"/>
       <c r="D4" s="22"/>
@@ -1756,10 +1648,10 @@
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>131</v>
+        <v>113</v>
       </c>
       <c r="C5" s="22"/>
       <c r="D5" s="22"/>
@@ -1767,10 +1659,10 @@
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>132</v>
+        <v>114</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>133</v>
+        <v>115</v>
       </c>
       <c r="C6" s="22"/>
       <c r="D6" s="22"/>
@@ -1778,12 +1670,12 @@
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="23" t="s">
-        <v>134</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="24" t="s">
-        <v>135</v>
+        <v>117</v>
       </c>
       <c r="B9" s="24"/>
       <c r="C9" s="24"/>

</xml_diff>

<commit_message>
fix: tampilkan '-' jika asset_condition null (tidak memaksa default string 'ADA')
</commit_message>
<xml_diff>
--- a/Dokumentasi_Spesifikasi_Mapping_Asset_Counting.xlsx
+++ b/Dokumentasi_Spesifikasi_Mapping_Asset_Counting.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="119">
   <si>
     <t>SPESIFIKASI MAPPING 1-TO-1 JSON KE EXCEL - FORM ASSET COUNTING</t>
   </si>
@@ -249,10 +249,10 @@
     <t>asset_condition</t>
   </si>
   <si>
-    <t>ADA</t>
-  </si>
-  <si>
-    <t>Status keberadaan barang (Highlight Kuning #FFFF00, default: ADA)</t>
+    <t>ADA / BAIK / RUSAK / null</t>
+  </si>
+  <si>
+    <t>Kondisi barang hasil cek (Jika null tampil -, Cell Kuning #FFFF00)</t>
   </si>
   <si>
     <t>Kolom K</t>
@@ -306,6 +306,9 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>ADA</t>
   </si>
   <si>
     <t>[Foto Unit Disematkan]</t>
@@ -1438,10 +1441,10 @@
         <v>96</v>
       </c>
       <c r="J6" s="17" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="K6" s="16" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L6" s="18" t="s">
         <v>89</v>
@@ -1452,13 +1455,13 @@
         <v>2</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E7" s="16" t="s">
         <v>96</v>
@@ -1476,7 +1479,7 @@
         <v>96</v>
       </c>
       <c r="J7" s="17" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="K7" s="16" t="s">
         <v>96</v>
@@ -1490,16 +1493,16 @@
         <v>3</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F8" s="19">
         <v>10346600</v>
@@ -1514,10 +1517,10 @@
         <v>73</v>
       </c>
       <c r="J8" s="17" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="K8" s="16" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L8" s="18" t="s">
         <v>89</v>
@@ -1528,13 +1531,13 @@
         <v>4</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E9" s="16" t="s">
         <v>96</v>
@@ -1552,7 +1555,7 @@
         <v>96</v>
       </c>
       <c r="J9" s="17" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="K9" s="16" t="s">
         <v>96</v>
@@ -1566,13 +1569,13 @@
         <v>5</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E10" s="16" t="s">
         <v>96</v>
@@ -1590,7 +1593,7 @@
         <v>96</v>
       </c>
       <c r="J10" s="17" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="K10" s="16" t="s">
         <v>96</v>
@@ -1617,7 +1620,7 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="20" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -1626,10 +1629,10 @@
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C3" s="22"/>
       <c r="D3" s="22"/>
@@ -1637,10 +1640,10 @@
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="21" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C4" s="22"/>
       <c r="D4" s="22"/>
@@ -1648,10 +1651,10 @@
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C5" s="22"/>
       <c r="D5" s="22"/>
@@ -1659,10 +1662,10 @@
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C6" s="22"/>
       <c r="D6" s="22"/>
@@ -1670,12 +1673,12 @@
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="23" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="24" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B9" s="24"/>
       <c r="C9" s="24"/>

</xml_diff>

<commit_message>
style: ubah semua header Form Asset Counting menjadi biru seragam dan hilangkan warna latar sel data
</commit_message>
<xml_diff>
--- a/Dokumentasi_Spesifikasi_Mapping_Asset_Counting.xlsx
+++ b/Dokumentasi_Spesifikasi_Mapping_Asset_Counting.xlsx
@@ -147,7 +147,7 @@
     <t>serial</t>
   </si>
   <si>
-    <t>Nomor barcode hasil scan fisik (Highlight Kuning #FFFF00)</t>
+    <t>Nomor barcode hasil scan fisik</t>
   </si>
   <si>
     <t>Kolom D</t>
@@ -252,7 +252,7 @@
     <t>ADA / BAIK / RUSAK / null</t>
   </si>
   <si>
-    <t>Kondisi barang hasil cek (Jika null tampil -, Cell Kuning #FFFF00)</t>
+    <t>Kondisi barang hasil cek (Jika null tampil -)</t>
   </si>
   <si>
     <t>Kolom K</t>
@@ -308,25 +308,25 @@
     <t>-</t>
   </si>
   <si>
+    <t>[Foto Unit Disematkan]</t>
+  </si>
+  <si>
+    <t>30200B1502001</t>
+  </si>
+  <si>
+    <t>RENOVASI BANGUNAN GEDUNG</t>
+  </si>
+  <si>
+    <t>30200K0302001</t>
+  </si>
+  <si>
+    <t>NOUVO</t>
+  </si>
+  <si>
+    <t>2014-07-18</t>
+  </si>
+  <si>
     <t>ADA</t>
-  </si>
-  <si>
-    <t>[Foto Unit Disematkan]</t>
-  </si>
-  <si>
-    <t>30200B1502001</t>
-  </si>
-  <si>
-    <t>RENOVASI BANGUNAN GEDUNG</t>
-  </si>
-  <si>
-    <t>30200K0302001</t>
-  </si>
-  <si>
-    <t>NOUVO</t>
-  </si>
-  <si>
-    <t>2014-07-18</t>
   </si>
   <si>
     <t>30200K1502001</t>
@@ -475,7 +475,7 @@
       <name val="Consolas"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -495,11 +495,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF8FAFC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -555,7 +550,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -593,13 +588,7 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -614,7 +603,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1387,16 +1376,16 @@
       <c r="D5" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="E5" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="F5" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="G5" s="15" t="s">
+      <c r="G5" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="H5" s="15" t="s">
+      <c r="H5" s="14" t="s">
         <v>67</v>
       </c>
       <c r="I5" s="14" t="s">
@@ -1413,192 +1402,192 @@
       </c>
     </row>
     <row r="6" ht="24" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" s="16">
+      <c r="A6" s="15">
         <v>1</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="16" t="s">
+      <c r="E6" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="F6" s="19">
+      <c r="F6" s="17">
         <v>2696351206</v>
       </c>
-      <c r="G6" s="19">
+      <c r="G6" s="17">
         <v>0</v>
       </c>
-      <c r="H6" s="19">
+      <c r="H6" s="17">
         <v>2696351206</v>
       </c>
-      <c r="I6" s="16" t="s">
+      <c r="I6" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="J6" s="17" t="s">
+      <c r="J6" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="K6" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="K6" s="16" t="s">
+      <c r="L6" s="16" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" s="15">
+        <v>2</v>
+      </c>
+      <c r="B7" s="15" t="s">
         <v>98</v>
       </c>
-      <c r="L6" s="18" t="s">
+      <c r="C7" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="F7" s="17">
+        <v>0</v>
+      </c>
+      <c r="G7" s="17">
+        <v>0</v>
+      </c>
+      <c r="H7" s="17">
+        <v>0</v>
+      </c>
+      <c r="I7" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="J7" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="K7" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="L7" s="16" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="7" ht="24" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" s="16">
-        <v>2</v>
-      </c>
-      <c r="B7" s="16" t="s">
-        <v>99</v>
-      </c>
-      <c r="C7" s="17" t="s">
-        <v>99</v>
-      </c>
-      <c r="D7" s="18" t="s">
+    <row r="8" ht="24" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="15">
+        <v>3</v>
+      </c>
+      <c r="B8" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="C8" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="F8" s="17">
+        <v>10346600</v>
+      </c>
+      <c r="G8" s="17">
+        <v>1939987</v>
+      </c>
+      <c r="H8" s="17">
+        <v>8406613</v>
+      </c>
+      <c r="I8" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="J8" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="K8" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="L8" s="16" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" s="15">
+        <v>4</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="E9" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="F7" s="19">
+      <c r="F9" s="17">
         <v>0</v>
       </c>
-      <c r="G7" s="19">
+      <c r="G9" s="17">
         <v>0</v>
       </c>
-      <c r="H7" s="19">
+      <c r="H9" s="17">
         <v>0</v>
       </c>
-      <c r="I7" s="16" t="s">
+      <c r="I9" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="J7" s="17" t="s">
-        <v>97</v>
-      </c>
-      <c r="K7" s="16" t="s">
+      <c r="J9" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="L7" s="18" t="s">
+      <c r="K9" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="L9" s="16" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="8" ht="24" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" s="16">
-        <v>3</v>
-      </c>
-      <c r="B8" s="16" t="s">
-        <v>101</v>
-      </c>
-      <c r="C8" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="D8" s="18" t="s">
-        <v>102</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>103</v>
-      </c>
-      <c r="F8" s="19">
-        <v>10346600</v>
-      </c>
-      <c r="G8" s="19">
-        <v>1939987</v>
-      </c>
-      <c r="H8" s="19">
-        <v>8406613</v>
-      </c>
-      <c r="I8" s="16" t="s">
-        <v>73</v>
-      </c>
-      <c r="J8" s="17" t="s">
-        <v>97</v>
-      </c>
-      <c r="K8" s="16" t="s">
-        <v>98</v>
-      </c>
-      <c r="L8" s="18" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" s="16">
-        <v>4</v>
-      </c>
-      <c r="B9" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="C9" s="17" t="s">
-        <v>104</v>
-      </c>
-      <c r="D9" s="18" t="s">
-        <v>105</v>
-      </c>
-      <c r="E9" s="16" t="s">
+    <row r="10" ht="24" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" s="15">
+        <v>5</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="E10" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="F9" s="19">
+      <c r="F10" s="17">
         <v>0</v>
       </c>
-      <c r="G9" s="19">
+      <c r="G10" s="17">
         <v>0</v>
       </c>
-      <c r="H9" s="19">
+      <c r="H10" s="17">
         <v>0</v>
       </c>
-      <c r="I9" s="16" t="s">
+      <c r="I10" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="J9" s="17" t="s">
-        <v>97</v>
-      </c>
-      <c r="K9" s="16" t="s">
+      <c r="J10" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="L9" s="18" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="10" ht="24" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" s="16">
-        <v>5</v>
-      </c>
-      <c r="B10" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>106</v>
-      </c>
-      <c r="D10" s="18" t="s">
-        <v>107</v>
-      </c>
-      <c r="E10" s="16" t="s">
+      <c r="K10" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="F10" s="19">
-        <v>0</v>
-      </c>
-      <c r="G10" s="19">
-        <v>0</v>
-      </c>
-      <c r="H10" s="19">
-        <v>0</v>
-      </c>
-      <c r="I10" s="16" t="s">
-        <v>96</v>
-      </c>
-      <c r="J10" s="17" t="s">
-        <v>97</v>
-      </c>
-      <c r="K10" s="16" t="s">
-        <v>96</v>
-      </c>
-      <c r="L10" s="18" t="s">
+      <c r="L10" s="16" t="s">
         <v>89</v>
       </c>
     </row>
@@ -1619,204 +1608,204 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="20" t="s">
         <v>112</v>
       </c>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="20" t="s">
         <v>114</v>
       </c>
-      <c r="C5" s="22"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="20" t="s">
         <v>116</v>
       </c>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="23" t="s">
+      <c r="A8" s="21" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="24" t="s">
+      <c r="A9" s="22" t="s">
         <v>118</v>
       </c>
-      <c r="B9" s="24"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
+      <c r="B9" s="22"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="24"/>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
+      <c r="A10" s="22"/>
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="24"/>
-      <c r="B11" s="24"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="24"/>
+      <c r="A11" s="22"/>
+      <c r="B11" s="22"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="24"/>
-      <c r="B12" s="24"/>
-      <c r="C12" s="24"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="24"/>
+      <c r="A12" s="22"/>
+      <c r="B12" s="22"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="24"/>
-      <c r="B13" s="24"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="24"/>
+      <c r="A13" s="22"/>
+      <c r="B13" s="22"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="24"/>
-      <c r="B14" s="24"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24"/>
+      <c r="A14" s="22"/>
+      <c r="B14" s="22"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="24"/>
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="24"/>
+      <c r="A15" s="22"/>
+      <c r="B15" s="22"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="24"/>
-      <c r="B16" s="24"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
+      <c r="A16" s="22"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="24"/>
-      <c r="B17" s="24"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
+      <c r="A17" s="22"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="24"/>
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
+      <c r="A18" s="22"/>
+      <c r="B18" s="22"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="24"/>
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
+      <c r="A19" s="22"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="24"/>
-      <c r="B20" s="24"/>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
+      <c r="A20" s="22"/>
+      <c r="B20" s="22"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="22"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="24"/>
-      <c r="B21" s="24"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
+      <c r="A21" s="22"/>
+      <c r="B21" s="22"/>
+      <c r="C21" s="22"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="22"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="24"/>
-      <c r="B22" s="24"/>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="24"/>
+      <c r="A22" s="22"/>
+      <c r="B22" s="22"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="22"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="24"/>
-      <c r="B23" s="24"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
+      <c r="A23" s="22"/>
+      <c r="B23" s="22"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="22"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="24"/>
-      <c r="B24" s="24"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
+      <c r="A24" s="22"/>
+      <c r="B24" s="22"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="22"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="24"/>
-      <c r="B25" s="24"/>
-      <c r="C25" s="24"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="24"/>
+      <c r="A25" s="22"/>
+      <c r="B25" s="22"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="22"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="24"/>
-      <c r="B26" s="24"/>
-      <c r="C26" s="24"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="24"/>
+      <c r="A26" s="22"/>
+      <c r="B26" s="22"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="22"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="24"/>
-      <c r="B27" s="24"/>
-      <c r="C27" s="24"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
+      <c r="A27" s="22"/>
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="22"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="24"/>
-      <c r="B28" s="24"/>
-      <c r="C28" s="24"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
+      <c r="A28" s="22"/>
+      <c r="B28" s="22"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>